<commit_message>
Pre-read the 30 final papers and draft the gap analysis
- pre_read_verification.csv: per-paper decisions from targeted full-text
  reading (keep/drop, split, duplicate risk, oversampling order, F1 type,
  statistical test, code, QA) with confidence levels
- 3 papers dropped as off-topic (R0014, R0615, R0072); 26 empirical kept
- gap_candidates.csv: verified k/N per gap + recommendation
- gap_analysis.md: main gap = evaluation leakage (duplicates 15/26 random
  splits, 0/26 grouped; oversampling before split 3/7), RQ proposal for v2.0
- workbook pre-fills the verification columns; humans confirm or edit
</commit_message>
<xml_diff>
--- a/literature/review/NCKH_FRNFR_VongCuoi.xlsx
+++ b/literature/review/NCKH_FRNFR_VongCuoi.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -493,46 +493,58 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Câu hỏi quan trọng nhất</t>
+          <t>Bản đọc trước (Claude)</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Mỗi bài: (1) chia train/test thế nào; (2) câu trùng có thể nằm ở cả train và test không; (3) oversampling / augmentation làm TRƯỚC hay SAU khi chia; (4) có kiểm định thống kê khi so model không; (5) báo loại F1 nào.</t>
+          <t>Các cột XÁC NHẬN và Q1–Q5 đã được Claude điền sẵn sau khi đọc các đoạn liên quan trong PDF (cột Ghi chú ghi độ chắc chắn). Người đọc chỉ cần mở PDF, kiểm tra nhanh các ô quan trọng (cách chia, câu trùng, oversampling, kiểm định) — ưu tiên dòng có độ chắc chắn 'thấp' / 'trung bình' — rồi ghi ĐỒNG Ý hoặc SỬA ở cột cuối. Số liệu gap chỉ tính các dòng đã có người ĐỒNG Ý / SỬA.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Bài lạc đề</t>
+          <t>Câu hỏi quan trọng nhất</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Nếu đọc thấy bài không phải phân loại yêu cầu FR/NFR: ghi 'Giữ?' = N và lý do ở Ghi chú. Không cần điền tiếp.</t>
+          <t>Mỗi bài: (1) chia train/test thế nào; (2) câu trùng có thể nằm ở cả train và test không; (3) oversampling / augmentation làm TRƯỚC hay SAU khi chia; (4) có kiểm định thống kê khi so model không; (5) báo loại F1 nào.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>QA Q1–Q5</t>
+          <t>Bài lạc đề</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>0/1/2 mỗi tiêu chí: Q1 mục tiêu rõ · Q2 dataset mô tả và truy cập được · Q3 đánh giá chặt chẽ (cách chia rõ, không rò rỉ hiển nhiên) · Q4 kết quả đủ (metric phù hợp, có độ biến thiên) · Q5 nêu hạn chế + tái lập được. Tổng ≥ 6 = tổng hợp chính.</t>
+          <t>Nếu đọc thấy bài không phải phân loại yêu cầu FR/NFR: ghi 'Giữ?' = N và lý do ở Ghi chú. Không cần điền tiếp.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
+          <t>QA Q1–Q5</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>0/1/2 mỗi tiêu chí: Q1 mục tiêu rõ · Q2 dataset mô tả và truy cập được · Q3 đánh giá chặt chẽ (cách chia rõ, không rò rỉ hiển nhiên) · Q4 kết quả đủ (metric phù hợp, có độ biến thiên) · Q5 nêu hạn chế + tái lập được. Tổng ≥ 6 = tổng hợp chính.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
           <t>Gap</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>Tab GD3_Gap đã có 7 gap ứng viên với số liệu SƠ BỘ. Sau khi đọc xong, điền cột 'Xác nhận sau khi đọc' bằng số thật (k/N) rồi họp chọn.</t>
         </is>
@@ -549,7 +561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ31"/>
+  <dimension ref="A1:AK31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -588,6 +600,7 @@
     <col width="16" customWidth="1" min="34" max="34"/>
     <col width="16" customWidth="1" min="35" max="35"/>
     <col width="16" customWidth="1" min="36" max="36"/>
+    <col width="16" customWidth="1" min="37" max="37"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -771,6 +784,11 @@
           <t>Ghi chú</t>
         </is>
       </c>
+      <c r="AK1" s="4" t="inlineStr">
+        <is>
+          <t>Người kiểm tra: ĐỒNG Ý / SỬA (ghi ô đã sửa)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -850,28 +868,72 @@
         </is>
       </c>
       <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
-      <c r="Y2" t="inlineStr"/>
-      <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr"/>
-      <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="inlineStr"/>
-      <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Corpus code (không phải yêu cầu)</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>Y (GitHub)</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>câu trùng làm thổi phồng metric tới 100%</t>
+        </is>
+      </c>
       <c r="AH2">
         <f>IF(COUNT(AC2:AG2)=5,SUM(AC2:AG2),"")</f>
         <v/>
       </c>
       <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr"/>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>Bài nền tảng cho G1 · Claude đọc (độ chắc chắn: cao)</t>
+        </is>
+      </c>
+      <c r="AK2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -943,28 +1005,87 @@
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr"/>
-      <c r="Y3" t="inlineStr"/>
-      <c r="Z3" t="inlineStr"/>
-      <c r="AA3" t="inlineStr"/>
-      <c r="AB3" t="inlineStr"/>
-      <c r="AC3" t="inlineStr"/>
-      <c r="AD3" t="inlineStr"/>
-      <c r="AE3" t="inlineStr"/>
-      <c r="AF3" t="inlineStr"/>
-      <c r="AG3" t="inlineStr"/>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Dataset riêng IoT healthcare (104 yêu cầu, 8 lớp)</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>multi-class (gồm Functional)</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Hybrid KNN + luật</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>không rõ</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>không rõ</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>không dùng</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>chỉ accuracy</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>accuracy 75,9–85%</t>
+        </is>
+      </c>
+      <c r="AC3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG3" t="n">
+        <v>1</v>
+      </c>
       <c r="AH3">
         <f>IF(COUNT(AC3:AG3)=5,SUM(AC3:AG3),"")</f>
         <v/>
       </c>
       <c r="AI3" t="inlineStr"/>
-      <c r="AJ3" t="inlineStr"/>
+      <c r="AJ3" t="inlineStr">
+        <is>
+          <t>Dataset rất nhỏ; nhóm ensemble nhưng thực chất là lai KNN + luật · Claude đọc (độ chắc chắn: trung bình)</t>
+        </is>
+      </c>
+      <c r="AK3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1036,28 +1157,87 @@
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
-      <c r="Y4" t="inlineStr"/>
-      <c r="Z4" t="inlineStr"/>
-      <c r="AA4" t="inlineStr"/>
-      <c r="AB4" t="inlineStr"/>
-      <c r="AC4" t="inlineStr"/>
-      <c r="AD4" t="inlineStr"/>
-      <c r="AE4" t="inlineStr"/>
-      <c r="AF4" t="inlineStr"/>
-      <c r="AG4" t="inlineStr"/>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Dataset riêng 600 câu FR (domain bảo hiểm)</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>multi-class (11 lớp FR)</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Weighted voting ensemble (accuracy làm trọng số)</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>70/30 phân tầng, một lần</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>không rõ</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>không dùng</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>chủ yếu accuracy</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>accuracy 79,8% (TF-IDF)</t>
+        </is>
+      </c>
+      <c r="AC4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG4" t="n">
+        <v>0</v>
+      </c>
       <c r="AH4">
         <f>IF(COUNT(AC4:AG4)=5,SUM(AC4:AG4),"")</f>
         <v/>
       </c>
       <c r="AI4" t="inlineStr"/>
-      <c r="AJ4" t="inlineStr"/>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>Phân loại FR con, không phải FR/NFR · Claude đọc (độ chắc chắn: trung bình)</t>
+        </is>
+      </c>
+      <c r="AK4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1137,28 +1317,87 @@
           <t>Xử lý mất cân bằng</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr"/>
-      <c r="X5" t="inlineStr"/>
-      <c r="Y5" t="inlineStr"/>
-      <c r="Z5" t="inlineStr"/>
-      <c r="AA5" t="inlineStr"/>
-      <c r="AB5" t="inlineStr"/>
-      <c r="AC5" t="inlineStr"/>
-      <c r="AD5" t="inlineStr"/>
-      <c r="AE5" t="inlineStr"/>
-      <c r="AF5" t="inlineStr"/>
-      <c r="AG5" t="inlineStr"/>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Dataset riêng + PROMISE</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>binary FR/NFR + multi-label con</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Ensemble BERT/DistilBERT/RoBERTa + attention fusion</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>35/35/30 ngẫu nhiên; 5-fold</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>Y (chia ngẫu nhiên, không khử trùng)</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>Y (dấu hiệu: oversampling để cân bằng dataset rồi mới chia)</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>F1 + accuracy</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>Y (paired t-test 10 lần chạy)</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>accuracy 95%, F1 0,94</t>
+        </is>
+      </c>
+      <c r="AC5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG5" t="n">
+        <v>1</v>
+      </c>
       <c r="AH5">
         <f>IF(COUNT(AC5:AG5)=5,SUM(AC5:AG5),"")</f>
         <v/>
       </c>
       <c r="AI5" t="inlineStr"/>
-      <c r="AJ5" t="inlineStr"/>
+      <c r="AJ5" t="inlineStr">
+        <is>
+          <t>Cần đọc kỹ đoạn oversampling để chắc thứ tự · Claude đọc (độ chắc chắn: trung bình)</t>
+        </is>
+      </c>
+      <c r="AK5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1230,28 +1469,87 @@
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr"/>
-      <c r="W6" t="inlineStr"/>
-      <c r="X6" t="inlineStr"/>
-      <c r="Y6" t="inlineStr"/>
-      <c r="Z6" t="inlineStr"/>
-      <c r="AA6" t="inlineStr"/>
-      <c r="AB6" t="inlineStr"/>
-      <c r="AC6" t="inlineStr"/>
-      <c r="AD6" t="inlineStr"/>
-      <c r="AE6" t="inlineStr"/>
-      <c r="AF6" t="inlineStr"/>
-      <c r="AG6" t="inlineStr"/>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>PURE</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>binary FR/NFR</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>CNN, LSTM, BiLSTM (DL)</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>80/20 một lần</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>Y (chia ngẫu nhiên, không khử trùng)</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>không dùng</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>P/R/F1 (không rõ loại)</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>BiLSTM tốt nhất về P/R/F1</t>
+        </is>
+      </c>
+      <c r="AC6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>0</v>
+      </c>
       <c r="AH6">
         <f>IF(COUNT(AC6:AG6)=5,SUM(AC6:AG6),"")</f>
         <v/>
       </c>
       <c r="AI6" t="inlineStr"/>
-      <c r="AJ6" t="inlineStr"/>
+      <c r="AJ6" t="inlineStr">
+        <is>
+          <t>Xếp nhóm ensemble do từ khóa; thực chất là so sánh DL · Claude đọc (độ chắc chắn: trung bình)</t>
+        </is>
+      </c>
+      <c r="AK6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1331,28 +1629,87 @@
           <t>Xử lý mất cân bằng</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr"/>
-      <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr"/>
-      <c r="V7" t="inlineStr"/>
-      <c r="W7" t="inlineStr"/>
-      <c r="X7" t="inlineStr"/>
-      <c r="Y7" t="inlineStr"/>
-      <c r="Z7" t="inlineStr"/>
-      <c r="AA7" t="inlineStr"/>
-      <c r="AB7" t="inlineStr"/>
-      <c r="AC7" t="inlineStr"/>
-      <c r="AD7" t="inlineStr"/>
-      <c r="AE7" t="inlineStr"/>
-      <c r="AF7" t="inlineStr"/>
-      <c r="AG7" t="inlineStr"/>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>PROMISE + 266 câu FR</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>binary + multi-class (17 lớp)</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>Ensemble DL (LSTM, BiLSTM, GRU, CNN) theo trọng số accuracy</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>35/35/30 cố định</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>Y (chia ngẫu nhiên, không khử trùng)</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>N (random oversampling trên tập train)</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>F1 + accuracy</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>accuracy 95,7% (binary), 93,4% (multi)</t>
+        </is>
+      </c>
+      <c r="AC7" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG7" t="n">
+        <v>0</v>
+      </c>
       <c r="AH7">
         <f>IF(COUNT(AC7:AG7)=5,SUM(AC7:AG7),"")</f>
         <v/>
       </c>
       <c r="AI7" t="inlineStr"/>
-      <c r="AJ7" t="inlineStr"/>
+      <c r="AJ7" t="inlineStr">
+        <is>
+          <t>Claude đọc (độ chắc chắn: trung bình)</t>
+        </is>
+      </c>
+      <c r="AK7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1432,28 +1789,87 @@
           <t>Xử lý mất cân bằng</t>
         </is>
       </c>
-      <c r="R8" t="inlineStr"/>
-      <c r="S8" t="inlineStr"/>
-      <c r="T8" t="inlineStr"/>
-      <c r="U8" t="inlineStr"/>
-      <c r="V8" t="inlineStr"/>
-      <c r="W8" t="inlineStr"/>
-      <c r="X8" t="inlineStr"/>
-      <c r="Y8" t="inlineStr"/>
-      <c r="Z8" t="inlineStr"/>
-      <c r="AA8" t="inlineStr"/>
-      <c r="AB8" t="inlineStr"/>
-      <c r="AC8" t="inlineStr"/>
-      <c r="AD8" t="inlineStr"/>
-      <c r="AE8" t="inlineStr"/>
-      <c r="AF8" t="inlineStr"/>
-      <c r="AG8" t="inlineStr"/>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>PROMISE (625) + PURE</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>binary FR/NFR + 6 lớp NFR</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>BERT + SVM/RF weighted voting</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>80/10/10 phân tầng, nhiều lần chia ngẫu nhiên</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>Y (chia ngẫu nhiên, không khử trùng)</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>không dùng</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>F1 + accuracy</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>Y (paired t-test)</t>
+        </is>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>F1 94,1% (binary)</t>
+        </is>
+      </c>
+      <c r="AC8" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF8" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG8" t="n">
+        <v>1</v>
+      </c>
       <c r="AH8">
         <f>IF(COUNT(AC8:AG8)=5,SUM(AC8:AG8),"")</f>
         <v/>
       </c>
       <c r="AI8" t="inlineStr"/>
-      <c r="AJ8" t="inlineStr"/>
+      <c r="AJ8" t="inlineStr">
+        <is>
+          <t>Ghi PURE 969 yêu cầu, có vẻ nhầm với PROMISE_exp · Claude đọc (độ chắc chắn: trung bình)</t>
+        </is>
+      </c>
+      <c r="AK8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1533,28 +1949,87 @@
           <t>Xử lý mất cân bằng</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr"/>
-      <c r="S9" t="inlineStr"/>
-      <c r="T9" t="inlineStr"/>
-      <c r="U9" t="inlineStr"/>
-      <c r="V9" t="inlineStr"/>
-      <c r="W9" t="inlineStr"/>
-      <c r="X9" t="inlineStr"/>
-      <c r="Y9" t="inlineStr"/>
-      <c r="Z9" t="inlineStr"/>
-      <c r="AA9" t="inlineStr"/>
-      <c r="AB9" t="inlineStr"/>
-      <c r="AC9" t="inlineStr"/>
-      <c r="AD9" t="inlineStr"/>
-      <c r="AE9" t="inlineStr"/>
-      <c r="AF9" t="inlineStr"/>
-      <c r="AG9" t="inlineStr"/>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>PROMISE_exp (969, 12 lớp)</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>multi-class (12 lớp)</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>SVM, LR, KNN, NB + Voting; hybrid SVM–BiLSTM</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>10-fold phân tầng</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>Y (chia ngẫu nhiên, không khử trùng)</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>Y (Hình 2 là phân bố lớp của dataset sau oversampling, rồi mới 10-fold)</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>P/R/F1 + accuracy</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>accuracy 98,79%</t>
+        </is>
+      </c>
+      <c r="AC9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG9" t="n">
+        <v>0</v>
+      </c>
       <c r="AH9">
         <f>IF(COUNT(AC9:AG9)=5,SUM(AC9:AG9),"")</f>
         <v/>
       </c>
       <c r="AI9" t="inlineStr"/>
-      <c r="AJ9" t="inlineStr"/>
+      <c r="AJ9" t="inlineStr">
+        <is>
+          <t>Ví dụ rõ nhất cho G2 · Claude đọc (độ chắc chắn: cao)</t>
+        </is>
+      </c>
+      <c r="AK9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1622,28 +2097,87 @@
       </c>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
-      <c r="S10" t="inlineStr"/>
-      <c r="T10" t="inlineStr"/>
-      <c r="U10" t="inlineStr"/>
-      <c r="V10" t="inlineStr"/>
-      <c r="W10" t="inlineStr"/>
-      <c r="X10" t="inlineStr"/>
-      <c r="Y10" t="inlineStr"/>
-      <c r="Z10" t="inlineStr"/>
-      <c r="AA10" t="inlineStr"/>
-      <c r="AB10" t="inlineStr"/>
-      <c r="AC10" t="inlineStr"/>
-      <c r="AD10" t="inlineStr"/>
-      <c r="AE10" t="inlineStr"/>
-      <c r="AF10" t="inlineStr"/>
-      <c r="AG10" t="inlineStr"/>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>không rõ (có thể PROMISE)</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>binary FR/NFR</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>Random Forest vs Gradient Boosting</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>không rõ (lặp 5 lần mỗi n-gram)</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>không rõ</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>không dùng</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>chủ yếu accuracy</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>accuracy &gt; 70%</t>
+        </is>
+      </c>
+      <c r="AC10" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF10" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG10" t="n">
+        <v>0</v>
+      </c>
       <c r="AH10">
         <f>IF(COUNT(AC10:AG10)=5,SUM(AC10:AG10),"")</f>
         <v/>
       </c>
       <c r="AI10" t="inlineStr"/>
-      <c r="AJ10" t="inlineStr"/>
+      <c r="AJ10" t="inlineStr">
+        <is>
+          <t>Claude đọc (độ chắc chắn: thấp)</t>
+        </is>
+      </c>
+      <c r="AK10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1719,28 +2253,87 @@
           <t>Xử lý mất cân bằng</t>
         </is>
       </c>
-      <c r="R11" t="inlineStr"/>
-      <c r="S11" t="inlineStr"/>
-      <c r="T11" t="inlineStr"/>
-      <c r="U11" t="inlineStr"/>
-      <c r="V11" t="inlineStr"/>
-      <c r="W11" t="inlineStr"/>
-      <c r="X11" t="inlineStr"/>
-      <c r="Y11" t="inlineStr"/>
-      <c r="Z11" t="inlineStr"/>
-      <c r="AA11" t="inlineStr"/>
-      <c r="AB11" t="inlineStr"/>
-      <c r="AC11" t="inlineStr"/>
-      <c r="AD11" t="inlineStr"/>
-      <c r="AE11" t="inlineStr"/>
-      <c r="AF11" t="inlineStr"/>
-      <c r="AG11" t="inlineStr"/>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>PROMISE + CCHIT</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>binary FR/NFR</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>FNRC (ensemble + mở rộng từ khóa)</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>70/10/20 một lần</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>Y (chia ngẫu nhiên, không khử trùng)</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>không dùng</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>F-measure</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>N (chỉ link dataset PROMISE)</t>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>F-measure 64%</t>
+        </is>
+      </c>
+      <c r="AC11" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD11" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG11" t="n">
+        <v>0</v>
+      </c>
       <c r="AH11">
         <f>IF(COUNT(AC11:AG11)=5,SUM(AC11:AG11),"")</f>
         <v/>
       </c>
       <c r="AI11" t="inlineStr"/>
-      <c r="AJ11" t="inlineStr"/>
+      <c r="AJ11" t="inlineStr">
+        <is>
+          <t>Claude đọc (độ chắc chắn: trung bình)</t>
+        </is>
+      </c>
+      <c r="AK11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1812,28 +2405,87 @@
       </c>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr"/>
-      <c r="S12" t="inlineStr"/>
-      <c r="T12" t="inlineStr"/>
-      <c r="U12" t="inlineStr"/>
-      <c r="V12" t="inlineStr"/>
-      <c r="W12" t="inlineStr"/>
-      <c r="X12" t="inlineStr"/>
-      <c r="Y12" t="inlineStr"/>
-      <c r="Z12" t="inlineStr"/>
-      <c r="AA12" t="inlineStr"/>
-      <c r="AB12" t="inlineStr"/>
-      <c r="AC12" t="inlineStr"/>
-      <c r="AD12" t="inlineStr"/>
-      <c r="AE12" t="inlineStr"/>
-      <c r="AF12" t="inlineStr"/>
-      <c r="AG12" t="inlineStr"/>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>PROMISE NFR (625, 15 project) + Stack Overflow</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>multi-class (12 lớp gồm F)</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>MNB, SVM, LR, DT, FCN (Keras)</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>repeated k-fold CV</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>Y (chia ngẫu nhiên, không khử trùng)</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>không dùng</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>P/R/F1 theo lớp + trung bình (không rõ loại)</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>Y (kiểm định khác biệt giữa 5 classifier)</t>
+        </is>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>MNB, SVM tốt nhất trên PROMISE</t>
+        </is>
+      </c>
+      <c r="AC12" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD12" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG12" t="n">
+        <v>1</v>
+      </c>
       <c r="AH12">
         <f>IF(COUNT(AC12:AG12)=5,SUM(AC12:AG12),"")</f>
         <v/>
       </c>
       <c r="AI12" t="inlineStr"/>
-      <c r="AJ12" t="inlineStr"/>
+      <c r="AJ12" t="inlineStr">
+        <is>
+          <t>Claude đọc (độ chắc chắn: trung bình)</t>
+        </is>
+      </c>
+      <c r="AK12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1909,7 +2561,11 @@
           <t>Xử lý mất cân bằng</t>
         </is>
       </c>
-      <c r="R13" t="inlineStr"/>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr"/>
       <c r="U13" t="inlineStr"/>
@@ -1920,17 +2576,17 @@
       <c r="Z13" t="inlineStr"/>
       <c r="AA13" t="inlineStr"/>
       <c r="AB13" t="inlineStr"/>
-      <c r="AC13" t="inlineStr"/>
-      <c r="AD13" t="inlineStr"/>
-      <c r="AE13" t="inlineStr"/>
-      <c r="AF13" t="inlineStr"/>
-      <c r="AG13" t="inlineStr"/>
       <c r="AH13">
         <f>IF(COUNT(AC13:AG13)=5,SUM(AC13:AG13),"")</f>
         <v/>
       </c>
       <c r="AI13" t="inlineStr"/>
-      <c r="AJ13" t="inlineStr"/>
+      <c r="AJ13" t="inlineStr">
+        <is>
+          <t>Lạc đề: phân loại review ứng dụng (tiếng Ả Rập), không phải đặc tả yêu cầu · Có augmentation dữ liệu · Claude đọc (độ chắc chắn: cao)</t>
+        </is>
+      </c>
+      <c r="AK13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2006,28 +2662,87 @@
           <t>Xử lý mất cân bằng</t>
         </is>
       </c>
-      <c r="R14" t="inlineStr"/>
-      <c r="S14" t="inlineStr"/>
-      <c r="T14" t="inlineStr"/>
-      <c r="U14" t="inlineStr"/>
-      <c r="V14" t="inlineStr"/>
-      <c r="W14" t="inlineStr"/>
-      <c r="X14" t="inlineStr"/>
-      <c r="Y14" t="inlineStr"/>
-      <c r="Z14" t="inlineStr"/>
-      <c r="AA14" t="inlineStr"/>
-      <c r="AB14" t="inlineStr"/>
-      <c r="AC14" t="inlineStr"/>
-      <c r="AD14" t="inlineStr"/>
-      <c r="AE14" t="inlineStr"/>
-      <c r="AF14" t="inlineStr"/>
-      <c r="AG14" t="inlineStr"/>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>PROMISE_exp (969)</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>multi-class (NFR)</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>15 classifier × 4 vectorizer (BoW, TF-IDF, Hashing, Chi2)</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>5-fold CV</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>Y (chia ngẫu nhiên, không khử trùng)</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>không dùng</t>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>F1 (không rõ loại)</t>
+        </is>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>LinearSVC + TF-IDF, F1 81,5%</t>
+        </is>
+      </c>
+      <c r="AC14" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD14" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG14" t="n">
+        <v>1</v>
+      </c>
       <c r="AH14">
         <f>IF(COUNT(AC14:AG14)=5,SUM(AC14:AG14),"")</f>
         <v/>
       </c>
       <c r="AI14" t="inlineStr"/>
-      <c r="AJ14" t="inlineStr"/>
+      <c r="AJ14" t="inlineStr">
+        <is>
+          <t>Claude đọc (độ chắc chắn: trung bình)</t>
+        </is>
+      </c>
+      <c r="AK14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2095,28 +2810,87 @@
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr"/>
-      <c r="S15" t="inlineStr"/>
-      <c r="T15" t="inlineStr"/>
-      <c r="U15" t="inlineStr"/>
-      <c r="V15" t="inlineStr"/>
-      <c r="W15" t="inlineStr"/>
-      <c r="X15" t="inlineStr"/>
-      <c r="Y15" t="inlineStr"/>
-      <c r="Z15" t="inlineStr"/>
-      <c r="AA15" t="inlineStr"/>
-      <c r="AB15" t="inlineStr"/>
-      <c r="AC15" t="inlineStr"/>
-      <c r="AD15" t="inlineStr"/>
-      <c r="AE15" t="inlineStr"/>
-      <c r="AF15" t="inlineStr"/>
-      <c r="AG15" t="inlineStr"/>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>PROMISE (NFR, 5 lớp)</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>multi-class (NFR)</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>BERT/RoBERTa + LoRA (prompt tuning)</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>80/20 + 10-fold CV (mô tả mâu thuẫn)</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>Y (chia ngẫu nhiên, không khử trùng)</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>không dùng</t>
+        </is>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>F1 (không rõ loại)</t>
+        </is>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AB15" t="inlineStr">
+        <is>
+          <t>RoBERTa-large F1 83,4%</t>
+        </is>
+      </c>
+      <c r="AC15" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD15" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG15" t="n">
+        <v>1</v>
+      </c>
       <c r="AH15">
         <f>IF(COUNT(AC15:AG15)=5,SUM(AC15:AG15),"")</f>
         <v/>
       </c>
       <c r="AI15" t="inlineStr"/>
-      <c r="AJ15" t="inlineStr"/>
+      <c r="AJ15" t="inlineStr">
+        <is>
+          <t>Có mục Threats to Validity · Claude đọc (độ chắc chắn: trung bình)</t>
+        </is>
+      </c>
+      <c r="AK15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2188,28 +2962,87 @@
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr"/>
-      <c r="S16" t="inlineStr"/>
-      <c r="T16" t="inlineStr"/>
-      <c r="U16" t="inlineStr"/>
-      <c r="V16" t="inlineStr"/>
-      <c r="W16" t="inlineStr"/>
-      <c r="X16" t="inlineStr"/>
-      <c r="Y16" t="inlineStr"/>
-      <c r="Z16" t="inlineStr"/>
-      <c r="AA16" t="inlineStr"/>
-      <c r="AB16" t="inlineStr"/>
-      <c r="AC16" t="inlineStr"/>
-      <c r="AD16" t="inlineStr"/>
-      <c r="AE16" t="inlineStr"/>
-      <c r="AF16" t="inlineStr"/>
-      <c r="AG16" t="inlineStr"/>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>PROMISE NFR</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>nhận diện NFR</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>Word2Vec + mở rộng từ khóa (gần không giám sát)</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>không chia (dựa trên độ tương đồng)</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>không áp dụng</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>không dùng (augmentation từ khóa, không phải oversampling)</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>P/R/F</t>
+        </is>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t>không nêu rõ trong đoạn đọc</t>
+        </is>
+      </c>
+      <c r="AC16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD16" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG16" t="n">
+        <v>0</v>
+      </c>
       <c r="AH16">
         <f>IF(COUNT(AC16:AG16)=5,SUM(AC16:AG16),"")</f>
         <v/>
       </c>
       <c r="AI16" t="inlineStr"/>
-      <c r="AJ16" t="inlineStr"/>
+      <c r="AJ16" t="inlineStr">
+        <is>
+          <t>Claude đọc (độ chắc chắn: thấp)</t>
+        </is>
+      </c>
+      <c r="AK16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2289,28 +3122,87 @@
         </is>
       </c>
       <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr"/>
-      <c r="S17" t="inlineStr"/>
-      <c r="T17" t="inlineStr"/>
-      <c r="U17" t="inlineStr"/>
-      <c r="V17" t="inlineStr"/>
-      <c r="W17" t="inlineStr"/>
-      <c r="X17" t="inlineStr"/>
-      <c r="Y17" t="inlineStr"/>
-      <c r="Z17" t="inlineStr"/>
-      <c r="AA17" t="inlineStr"/>
-      <c r="AB17" t="inlineStr"/>
-      <c r="AC17" t="inlineStr"/>
-      <c r="AD17" t="inlineStr"/>
-      <c r="AE17" t="inlineStr"/>
-      <c r="AF17" t="inlineStr"/>
-      <c r="AG17" t="inlineStr"/>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>PROMISE (625)</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>binary FR/NFR + NFR</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>NB, kNN, LDA… + tiền xử lý chuẩn hóa</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>10-fold CV; 5 × 5-fold</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>Y (chia ngẫu nhiên, không khử trùng)</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>không dùng</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>weighted P/R</t>
+        </is>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>N (p-value chỉ cho accuracy, không so model)</t>
+        </is>
+      </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t>tăng 4,48% nhờ tiền xử lý</t>
+        </is>
+      </c>
+      <c r="AC17" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD17" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG17" t="n">
+        <v>1</v>
+      </c>
       <c r="AH17">
         <f>IF(COUNT(AC17:AG17)=5,SUM(AC17:AG17),"")</f>
         <v/>
       </c>
       <c r="AI17" t="inlineStr"/>
-      <c r="AJ17" t="inlineStr"/>
+      <c r="AJ17" t="inlineStr">
+        <is>
+          <t>Bài duy nhất tách riêng ảnh hưởng tiền xử lý (G7) · Claude đọc (độ chắc chắn: cao)</t>
+        </is>
+      </c>
+      <c r="AK17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2378,28 +3270,87 @@
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr"/>
-      <c r="S18" t="inlineStr"/>
-      <c r="T18" t="inlineStr"/>
-      <c r="U18" t="inlineStr"/>
-      <c r="V18" t="inlineStr"/>
-      <c r="W18" t="inlineStr"/>
-      <c r="X18" t="inlineStr"/>
-      <c r="Y18" t="inlineStr"/>
-      <c r="Z18" t="inlineStr"/>
-      <c r="AA18" t="inlineStr"/>
-      <c r="AB18" t="inlineStr"/>
-      <c r="AC18" t="inlineStr"/>
-      <c r="AD18" t="inlineStr"/>
-      <c r="AE18" t="inlineStr"/>
-      <c r="AF18" t="inlineStr"/>
-      <c r="AG18" t="inlineStr"/>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>PROMISE + PURE</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>binary FR/NFR</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>LR, SVM, DT, RF, MLP</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>không rõ</t>
+        </is>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>không rõ</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>không dùng</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>chủ yếu accuracy</t>
+        </is>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AB18" t="inlineStr">
+        <is>
+          <t>không nêu rõ trong đoạn đọc</t>
+        </is>
+      </c>
+      <c r="AC18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG18" t="n">
+        <v>0</v>
+      </c>
       <c r="AH18">
         <f>IF(COUNT(AC18:AG18)=5,SUM(AC18:AG18),"")</f>
         <v/>
       </c>
       <c r="AI18" t="inlineStr"/>
-      <c r="AJ18" t="inlineStr"/>
+      <c r="AJ18" t="inlineStr">
+        <is>
+          <t>Claude đọc (độ chắc chắn: thấp)</t>
+        </is>
+      </c>
+      <c r="AK18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2471,28 +3422,87 @@
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr"/>
-      <c r="S19" t="inlineStr"/>
-      <c r="T19" t="inlineStr"/>
-      <c r="U19" t="inlineStr"/>
-      <c r="V19" t="inlineStr"/>
-      <c r="W19" t="inlineStr"/>
-      <c r="X19" t="inlineStr"/>
-      <c r="Y19" t="inlineStr"/>
-      <c r="Z19" t="inlineStr"/>
-      <c r="AA19" t="inlineStr"/>
-      <c r="AB19" t="inlineStr"/>
-      <c r="AC19" t="inlineStr"/>
-      <c r="AD19" t="inlineStr"/>
-      <c r="AE19" t="inlineStr"/>
-      <c r="AF19" t="inlineStr"/>
-      <c r="AG19" t="inlineStr"/>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>PURE</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>binary FR/NFR</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>So sánh trích xuất đặc trưng (BoW, TF-IDF) + ML</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>không rõ</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>không rõ</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>không dùng</t>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>chủ yếu accuracy</t>
+        </is>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AB19" t="inlineStr">
+        <is>
+          <t>chênh 3,84% giữa hai kỹ thuật</t>
+        </is>
+      </c>
+      <c r="AC19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG19" t="n">
+        <v>0</v>
+      </c>
       <c r="AH19">
         <f>IF(COUNT(AC19:AG19)=5,SUM(AC19:AG19),"")</f>
         <v/>
       </c>
       <c r="AI19" t="inlineStr"/>
-      <c r="AJ19" t="inlineStr"/>
+      <c r="AJ19" t="inlineStr">
+        <is>
+          <t>Claude đọc (độ chắc chắn: thấp)</t>
+        </is>
+      </c>
+      <c r="AK19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2568,28 +3578,87 @@
         </is>
       </c>
       <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="inlineStr"/>
-      <c r="S20" t="inlineStr"/>
-      <c r="T20" t="inlineStr"/>
-      <c r="U20" t="inlineStr"/>
-      <c r="V20" t="inlineStr"/>
-      <c r="W20" t="inlineStr"/>
-      <c r="X20" t="inlineStr"/>
-      <c r="Y20" t="inlineStr"/>
-      <c r="Z20" t="inlineStr"/>
-      <c r="AA20" t="inlineStr"/>
-      <c r="AB20" t="inlineStr"/>
-      <c r="AC20" t="inlineStr"/>
-      <c r="AD20" t="inlineStr"/>
-      <c r="AE20" t="inlineStr"/>
-      <c r="AF20" t="inlineStr"/>
-      <c r="AG20" t="inlineStr"/>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>PROMISE NFR</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>binary FR/NFR + multi-class</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>Zero-shot learning (mô hình ngôn ngữ)</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>không huấn luyện (zero-shot); baseline 10-fold</t>
+        </is>
+      </c>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>không áp dụng</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>không dùng</t>
+        </is>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>weighted F1 + theo lớp</t>
+        </is>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>Y (ANOVA + Friedman)</t>
+        </is>
+      </c>
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>Một phần (model BERT4RE trên Zenodo)</t>
+        </is>
+      </c>
+      <c r="AB20" t="inlineStr">
+        <is>
+          <t>F1 0,66–0,80</t>
+        </is>
+      </c>
+      <c r="AC20" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD20" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE20" t="n">
+        <v>2</v>
+      </c>
+      <c r="AF20" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG20" t="n">
+        <v>1</v>
+      </c>
       <c r="AH20">
         <f>IF(COUNT(AC20:AG20)=5,SUM(AC20:AG20),"")</f>
         <v/>
       </c>
       <c r="AI20" t="inlineStr"/>
-      <c r="AJ20" t="inlineStr"/>
+      <c r="AJ20" t="inlineStr">
+        <is>
+          <t>Claude đọc (độ chắc chắn: cao)</t>
+        </is>
+      </c>
+      <c r="AK20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2669,28 +3738,87 @@
           <t>Xử lý mất cân bằng</t>
         </is>
       </c>
-      <c r="R21" t="inlineStr"/>
-      <c r="S21" t="inlineStr"/>
-      <c r="T21" t="inlineStr"/>
-      <c r="U21" t="inlineStr"/>
-      <c r="V21" t="inlineStr"/>
-      <c r="W21" t="inlineStr"/>
-      <c r="X21" t="inlineStr"/>
-      <c r="Y21" t="inlineStr"/>
-      <c r="Z21" t="inlineStr"/>
-      <c r="AA21" t="inlineStr"/>
-      <c r="AB21" t="inlineStr"/>
-      <c r="AC21" t="inlineStr"/>
-      <c r="AD21" t="inlineStr"/>
-      <c r="AE21" t="inlineStr"/>
-      <c r="AF21" t="inlineStr"/>
-      <c r="AG21" t="inlineStr"/>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>PROMISE + SecReq (ePurse)</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>binary FR/NFR</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>SVM, CNN, FastText+SVM, FastText+CNN</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>70/30 holdout</t>
+        </is>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>Y (chia ngẫu nhiên, không khử trùng)</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>Y (dấu hiệu: nhân bản từng lớp trên dataset rồi mới chia)</t>
+        </is>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>F1 + accuracy</t>
+        </is>
+      </c>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AA21" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AB21" t="inlineStr">
+        <is>
+          <t>CNN accuracy 99% trên PROMISE</t>
+        </is>
+      </c>
+      <c r="AC21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG21" t="n">
+        <v>0</v>
+      </c>
       <c r="AH21">
         <f>IF(COUNT(AC21:AG21)=5,SUM(AC21:AG21),"")</f>
         <v/>
       </c>
       <c r="AI21" t="inlineStr"/>
-      <c r="AJ21" t="inlineStr"/>
+      <c r="AJ21" t="inlineStr">
+        <is>
+          <t>Accuracy 99% khớp với giả thuyết rò rỉ do nhân bản · Claude đọc (độ chắc chắn: trung bình)</t>
+        </is>
+      </c>
+      <c r="AK21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2774,28 +3902,87 @@
           <t>Xử lý mất cân bằng</t>
         </is>
       </c>
-      <c r="R22" t="inlineStr"/>
-      <c r="S22" t="inlineStr"/>
-      <c r="T22" t="inlineStr"/>
-      <c r="U22" t="inlineStr"/>
-      <c r="V22" t="inlineStr"/>
-      <c r="W22" t="inlineStr"/>
-      <c r="X22" t="inlineStr"/>
-      <c r="Y22" t="inlineStr"/>
-      <c r="Z22" t="inlineStr"/>
-      <c r="AA22" t="inlineStr"/>
-      <c r="AB22" t="inlineStr"/>
-      <c r="AC22" t="inlineStr"/>
-      <c r="AD22" t="inlineStr"/>
-      <c r="AE22" t="inlineStr"/>
-      <c r="AF22" t="inlineStr"/>
-      <c r="AG22" t="inlineStr"/>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>PROMISE + FR_NFR</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>binary FR/NFR + multi-class</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>BERT fine-tuning (khảo sát hyperparameter)</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>10-fold phân tầng</t>
+        </is>
+      </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>Y (chia ngẫu nhiên, không khử trùng)</t>
+        </is>
+      </c>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t>không dùng</t>
+        </is>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>F1 trung bình (không rõ loại)</t>
+        </is>
+      </c>
+      <c r="Z22" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>Y (GitHub)</t>
+        </is>
+      </c>
+      <c r="AB22" t="inlineStr">
+        <is>
+          <t>F1 0,99 (PROMISE), 0,97 (FR_NFR)</t>
+        </is>
+      </c>
+      <c r="AC22" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD22" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG22" t="n">
+        <v>2</v>
+      </c>
       <c r="AH22">
         <f>IF(COUNT(AC22:AG22)=5,SUM(AC22:AG22),"")</f>
         <v/>
       </c>
       <c r="AI22" t="inlineStr"/>
-      <c r="AJ22" t="inlineStr"/>
+      <c r="AJ22" t="inlineStr">
+        <is>
+          <t>F1 0,99 rất cao · Claude đọc (độ chắc chắn: cao)</t>
+        </is>
+      </c>
+      <c r="AK22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2855,28 +4042,72 @@
           <t>Xử lý mất cân bằng</t>
         </is>
       </c>
-      <c r="R23" t="inlineStr"/>
-      <c r="S23" t="inlineStr"/>
-      <c r="T23" t="inlineStr"/>
-      <c r="U23" t="inlineStr"/>
-      <c r="V23" t="inlineStr"/>
-      <c r="W23" t="inlineStr"/>
-      <c r="X23" t="inlineStr"/>
-      <c r="Y23" t="inlineStr"/>
-      <c r="Z23" t="inlineStr"/>
-      <c r="AA23" t="inlineStr"/>
-      <c r="AB23" t="inlineStr"/>
-      <c r="AC23" t="inlineStr"/>
-      <c r="AD23" t="inlineStr"/>
-      <c r="AE23" t="inlineStr"/>
-      <c r="AF23" t="inlineStr"/>
-      <c r="AG23" t="inlineStr"/>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>109 yêu cầu tiếng Tây Ban Nha</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="X23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Z23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>Y (Zenodo)</t>
+        </is>
+      </c>
+      <c r="AB23" t="inlineStr">
+        <is>
+          <t>Fleiss kappa 0,78</t>
+        </is>
+      </c>
       <c r="AH23">
         <f>IF(COUNT(AC23:AG23)=5,SUM(AC23:AG23),"")</f>
         <v/>
       </c>
       <c r="AI23" t="inlineStr"/>
-      <c r="AJ23" t="inlineStr"/>
+      <c r="AJ23" t="inlineStr">
+        <is>
+          <t>Không có thí nghiệm phân loại (bài xây dataset tiếng Tây Ban Nha) · Dùng được làm bài nền về tái lập / FAIR · Claude đọc (độ chắc chắn: cao)</t>
+        </is>
+      </c>
+      <c r="AK23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2960,28 +4191,87 @@
           <t>Xử lý mất cân bằng</t>
         </is>
       </c>
-      <c r="R24" t="inlineStr"/>
-      <c r="S24" t="inlineStr"/>
-      <c r="T24" t="inlineStr"/>
-      <c r="U24" t="inlineStr"/>
-      <c r="V24" t="inlineStr"/>
-      <c r="W24" t="inlineStr"/>
-      <c r="X24" t="inlineStr"/>
-      <c r="Y24" t="inlineStr"/>
-      <c r="Z24" t="inlineStr"/>
-      <c r="AA24" t="inlineStr"/>
-      <c r="AB24" t="inlineStr"/>
-      <c r="AC24" t="inlineStr"/>
-      <c r="AD24" t="inlineStr"/>
-      <c r="AE24" t="inlineStr"/>
-      <c r="AF24" t="inlineStr"/>
-      <c r="AG24" t="inlineStr"/>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>Dataset mới 9.529 FR từ 315 project (Zenodo)</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>multi-class (5 loại FR theo EARS)</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>SVM, KNN, DL</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>cross-project</t>
+        </is>
+      </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>N (chia theo project)</t>
+        </is>
+      </c>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>không rõ</t>
+        </is>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>P/R/F1</t>
+        </is>
+      </c>
+      <c r="Z24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>Y (Zenodo)</t>
+        </is>
+      </c>
+      <c r="AB24" t="inlineStr">
+        <is>
+          <t>SVM P/R/F1 0,90</t>
+        </is>
+      </c>
+      <c r="AC24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AF24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG24" t="n">
+        <v>2</v>
+      </c>
       <c r="AH24">
         <f>IF(COUNT(AC24:AG24)=5,SUM(AC24:AG24),"")</f>
         <v/>
       </c>
       <c r="AI24" t="inlineStr"/>
-      <c r="AJ24" t="inlineStr"/>
+      <c r="AJ24" t="inlineStr">
+        <is>
+          <t>Phân loại FR con, không phải FR/NFR; mạnh về tổng quát hóa · Claude đọc (độ chắc chắn: trung bình)</t>
+        </is>
+      </c>
+      <c r="AK24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3069,28 +4359,87 @@
           <t>Xử lý mất cân bằng</t>
         </is>
       </c>
-      <c r="R25" t="inlineStr"/>
-      <c r="S25" t="inlineStr"/>
-      <c r="T25" t="inlineStr"/>
-      <c r="U25" t="inlineStr"/>
-      <c r="V25" t="inlineStr"/>
-      <c r="W25" t="inlineStr"/>
-      <c r="X25" t="inlineStr"/>
-      <c r="Y25" t="inlineStr"/>
-      <c r="Z25" t="inlineStr"/>
-      <c r="AA25" t="inlineStr"/>
-      <c r="AB25" t="inlineStr"/>
-      <c r="AC25" t="inlineStr"/>
-      <c r="AD25" t="inlineStr"/>
-      <c r="AE25" t="inlineStr"/>
-      <c r="AF25" t="inlineStr"/>
-      <c r="AG25" t="inlineStr"/>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>PROMISE NFR + bản gán nhãn lại</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>binary FR/NFR + NFR</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>BERT (NoRBERT)</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>75/25 phân tầng; 10-fold phân tầng; leave-one-project-out</t>
+        </is>
+      </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>Một phần (có bỏ 1 câu trùng; nhắc PROMISE có câu trùng)</t>
+        </is>
+      </c>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>N (oversampling chỉ trên tập train)</t>
+        </is>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>weighted F1 + theo lớp</t>
+        </is>
+      </c>
+      <c r="Z25" t="inlineStr">
+        <is>
+          <t>Y (paired t-test)</t>
+        </is>
+      </c>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>Y (Zenodo)</t>
+        </is>
+      </c>
+      <c r="AB25" t="inlineStr">
+        <is>
+          <t>F1 tới 94%</t>
+        </is>
+      </c>
+      <c r="AC25" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD25" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE25" t="n">
+        <v>2</v>
+      </c>
+      <c r="AF25" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG25" t="n">
+        <v>2</v>
+      </c>
       <c r="AH25">
         <f>IF(COUNT(AC25:AG25)=5,SUM(AC25:AG25),"")</f>
         <v/>
       </c>
       <c r="AI25" t="inlineStr"/>
-      <c r="AJ25" t="inlineStr"/>
+      <c r="AJ25" t="inlineStr">
+        <is>
+          <t>Bài chuẩn nhất trong bộ · Claude đọc (độ chắc chắn: cao)</t>
+        </is>
+      </c>
+      <c r="AK25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3166,7 +4515,11 @@
           <t>Xử lý mất cân bằng</t>
         </is>
       </c>
-      <c r="R26" t="inlineStr"/>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr"/>
       <c r="U26" t="inlineStr"/>
@@ -3177,17 +4530,17 @@
       <c r="Z26" t="inlineStr"/>
       <c r="AA26" t="inlineStr"/>
       <c r="AB26" t="inlineStr"/>
-      <c r="AC26" t="inlineStr"/>
-      <c r="AD26" t="inlineStr"/>
-      <c r="AE26" t="inlineStr"/>
-      <c r="AF26" t="inlineStr"/>
-      <c r="AG26" t="inlineStr"/>
       <c r="AH26">
         <f>IF(COUNT(AC26:AG26)=5,SUM(AC26:AG26),"")</f>
         <v/>
       </c>
       <c r="AI26" t="inlineStr"/>
-      <c r="AJ26" t="inlineStr"/>
+      <c r="AJ26" t="inlineStr">
+        <is>
+          <t>Lạc đề: phân loại câu mơ hồ (clear vs ambiguous), không phải FR/NFR · Ví dụ làm đúng: SMOTE chỉ trên tập train · Claude đọc (độ chắc chắn: cao)</t>
+        </is>
+      </c>
+      <c r="AK26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3263,28 +4616,87 @@
           <t>Xử lý mất cân bằng</t>
         </is>
       </c>
-      <c r="R27" t="inlineStr"/>
-      <c r="S27" t="inlineStr"/>
-      <c r="T27" t="inlineStr"/>
-      <c r="U27" t="inlineStr"/>
-      <c r="V27" t="inlineStr"/>
-      <c r="W27" t="inlineStr"/>
-      <c r="X27" t="inlineStr"/>
-      <c r="Y27" t="inlineStr"/>
-      <c r="Z27" t="inlineStr"/>
-      <c r="AA27" t="inlineStr"/>
-      <c r="AB27" t="inlineStr"/>
-      <c r="AC27" t="inlineStr"/>
-      <c r="AD27" t="inlineStr"/>
-      <c r="AE27" t="inlineStr"/>
-      <c r="AF27" t="inlineStr"/>
-      <c r="AG27" t="inlineStr"/>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>PURE</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>multi-class (NFR)</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>SVM + ROS / SMOTE / các cách cân bằng</t>
+        </is>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>k-fold (so nhiều số fold)</t>
+        </is>
+      </c>
+      <c r="W27" t="inlineStr">
+        <is>
+          <t>Y (chia ngẫu nhiên, không khử trùng)</t>
+        </is>
+      </c>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t>không rõ (nghi trước khi chia: accuracy tăng 22–27%)</t>
+        </is>
+      </c>
+      <c r="Y27" t="inlineStr">
+        <is>
+          <t>F1 + accuracy</t>
+        </is>
+      </c>
+      <c r="Z27" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AA27" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AB27" t="inlineStr">
+        <is>
+          <t>accuracy +26,7% nhờ cân bằng lớp</t>
+        </is>
+      </c>
+      <c r="AC27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG27" t="n">
+        <v>0</v>
+      </c>
       <c r="AH27">
         <f>IF(COUNT(AC27:AG27)=5,SUM(AC27:AG27),"")</f>
         <v/>
       </c>
       <c r="AI27" t="inlineStr"/>
-      <c r="AJ27" t="inlineStr"/>
+      <c r="AJ27" t="inlineStr">
+        <is>
+          <t>Mức tăng lớn đáng ngờ · Claude đọc (độ chắc chắn: thấp)</t>
+        </is>
+      </c>
+      <c r="AK27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3368,28 +4780,87 @@
           <t>Xử lý mất cân bằng</t>
         </is>
       </c>
-      <c r="R28" t="inlineStr"/>
-      <c r="S28" t="inlineStr"/>
-      <c r="T28" t="inlineStr"/>
-      <c r="U28" t="inlineStr"/>
-      <c r="V28" t="inlineStr"/>
-      <c r="W28" t="inlineStr"/>
-      <c r="X28" t="inlineStr"/>
-      <c r="Y28" t="inlineStr"/>
-      <c r="Z28" t="inlineStr"/>
-      <c r="AA28" t="inlineStr"/>
-      <c r="AB28" t="inlineStr"/>
-      <c r="AC28" t="inlineStr"/>
-      <c r="AD28" t="inlineStr"/>
-      <c r="AE28" t="inlineStr"/>
-      <c r="AF28" t="inlineStr"/>
-      <c r="AG28" t="inlineStr"/>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>PROMISE NFR mở rộng (6.086, 5 domain)</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>binary FR/NFR</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>Đa phương thức + contrastive + domain adaptation</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>leave-one-domain-out (+ chia thường)</t>
+        </is>
+      </c>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>N (có đánh giá theo domain)</t>
+        </is>
+      </c>
+      <c r="X28" t="inlineStr">
+        <is>
+          <t>không dùng (augmentation cho contrastive)</t>
+        </is>
+      </c>
+      <c r="Y28" t="inlineStr">
+        <is>
+          <t>F1 + accuracy</t>
+        </is>
+      </c>
+      <c r="Z28" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AA28" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AB28" t="inlineStr">
+        <is>
+          <t>accuracy 95,8%, F1 95,4%</t>
+        </is>
+      </c>
+      <c r="AC28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG28" t="n">
+        <v>0</v>
+      </c>
       <c r="AH28">
         <f>IF(COUNT(AC28:AG28)=5,SUM(AC28:AG28),"")</f>
         <v/>
       </c>
       <c r="AI28" t="inlineStr"/>
-      <c r="AJ28" t="inlineStr"/>
+      <c r="AJ28" t="inlineStr">
+        <is>
+          <t>Venue chất lượng không rõ; chỉ ablation, không kiểm định · Claude đọc (độ chắc chắn: thấp)</t>
+        </is>
+      </c>
+      <c r="AK28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3469,28 +4940,87 @@
           <t>Xử lý mất cân bằng</t>
         </is>
       </c>
-      <c r="R29" t="inlineStr"/>
-      <c r="S29" t="inlineStr"/>
-      <c r="T29" t="inlineStr"/>
-      <c r="U29" t="inlineStr"/>
-      <c r="V29" t="inlineStr"/>
-      <c r="W29" t="inlineStr"/>
-      <c r="X29" t="inlineStr"/>
-      <c r="Y29" t="inlineStr"/>
-      <c r="Z29" t="inlineStr"/>
-      <c r="AA29" t="inlineStr"/>
-      <c r="AB29" t="inlineStr"/>
-      <c r="AC29" t="inlineStr"/>
-      <c r="AD29" t="inlineStr"/>
-      <c r="AE29" t="inlineStr"/>
-      <c r="AF29" t="inlineStr"/>
-      <c r="AG29" t="inlineStr"/>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>PROMISE + SecReq</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>binary FR/NFR + NFR + Sec</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>LLM prompting (GPT-4, Gemini, Llama…) so với fine-tuned</t>
+        </is>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>8:1:1 phân tầng, một lần</t>
+        </is>
+      </c>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>Y (chia ngẫu nhiên, không khử trùng)</t>
+        </is>
+      </c>
+      <c r="X29" t="inlineStr">
+        <is>
+          <t>không dùng</t>
+        </is>
+      </c>
+      <c r="Y29" t="inlineStr">
+        <is>
+          <t>macro-F1</t>
+        </is>
+      </c>
+      <c r="Z29" t="inlineStr">
+        <is>
+          <t>Y (Scott-Knott ESD)</t>
+        </is>
+      </c>
+      <c r="AA29" t="inlineStr">
+        <is>
+          <t>không rõ</t>
+        </is>
+      </c>
+      <c r="AB29" t="inlineStr">
+        <is>
+          <t>GPT-4 macro-F1 0,73 (Sec)</t>
+        </is>
+      </c>
+      <c r="AC29" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD29" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE29" t="n">
+        <v>2</v>
+      </c>
+      <c r="AF29" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG29" t="n">
+        <v>1</v>
+      </c>
       <c r="AH29">
         <f>IF(COUNT(AC29:AG29)=5,SUM(AC29:AG29),"")</f>
         <v/>
       </c>
       <c r="AI29" t="inlineStr"/>
-      <c r="AJ29" t="inlineStr"/>
+      <c r="AJ29" t="inlineStr">
+        <is>
+          <t>Claude đọc (độ chắc chắn: cao)</t>
+        </is>
+      </c>
+      <c r="AK29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3570,28 +5100,87 @@
           <t>Xử lý mất cân bằng</t>
         </is>
       </c>
-      <c r="R30" t="inlineStr"/>
-      <c r="S30" t="inlineStr"/>
-      <c r="T30" t="inlineStr"/>
-      <c r="U30" t="inlineStr"/>
-      <c r="V30" t="inlineStr"/>
-      <c r="W30" t="inlineStr"/>
-      <c r="X30" t="inlineStr"/>
-      <c r="Y30" t="inlineStr"/>
-      <c r="Z30" t="inlineStr"/>
-      <c r="AA30" t="inlineStr"/>
-      <c r="AB30" t="inlineStr"/>
-      <c r="AC30" t="inlineStr"/>
-      <c r="AD30" t="inlineStr"/>
-      <c r="AE30" t="inlineStr"/>
-      <c r="AF30" t="inlineStr"/>
-      <c r="AG30" t="inlineStr"/>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>PROMISE_exp (969)</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>multi-class (12 lớp)</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>LR, SVM… + SMOTE-Tomek</t>
+        </is>
+      </c>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>k-fold phân tầng</t>
+        </is>
+      </c>
+      <c r="W30" t="inlineStr">
+        <is>
+          <t>Y (chia ngẫu nhiên, không khử trùng)</t>
+        </is>
+      </c>
+      <c r="X30" t="inlineStr">
+        <is>
+          <t>N (SMOTE-Tomek trong từng fold)</t>
+        </is>
+      </c>
+      <c r="Y30" t="inlineStr">
+        <is>
+          <t>weighted F1 (recall = accuracy) + MCC</t>
+        </is>
+      </c>
+      <c r="Z30" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AA30" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AB30" t="inlineStr">
+        <is>
+          <t>LR accuracy 76,2% ± 2,6%</t>
+        </is>
+      </c>
+      <c r="AC30" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD30" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE30" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF30" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG30" t="n">
+        <v>1</v>
+      </c>
       <c r="AH30">
         <f>IF(COUNT(AC30:AG30)=5,SUM(AC30:AG30),"")</f>
         <v/>
       </c>
       <c r="AI30" t="inlineStr"/>
-      <c r="AJ30" t="inlineStr"/>
+      <c r="AJ30" t="inlineStr">
+        <is>
+          <t>Preprint arXiv (chưa bình duyệt) · Claude đọc (độ chắc chắn: trung bình)</t>
+        </is>
+      </c>
+      <c r="AK30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3675,28 +5264,87 @@
           <t>Xử lý mất cân bằng</t>
         </is>
       </c>
-      <c r="R31" t="inlineStr"/>
-      <c r="S31" t="inlineStr"/>
-      <c r="T31" t="inlineStr"/>
-      <c r="U31" t="inlineStr"/>
-      <c r="V31" t="inlineStr"/>
-      <c r="W31" t="inlineStr"/>
-      <c r="X31" t="inlineStr"/>
-      <c r="Y31" t="inlineStr"/>
-      <c r="Z31" t="inlineStr"/>
-      <c r="AA31" t="inlineStr"/>
-      <c r="AB31" t="inlineStr"/>
-      <c r="AC31" t="inlineStr"/>
-      <c r="AD31" t="inlineStr"/>
-      <c r="AE31" t="inlineStr"/>
-      <c r="AF31" t="inlineStr"/>
-      <c r="AG31" t="inlineStr"/>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>SecReq, DOSSPRE, PROMISE+</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>binary (security vs non-security)</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>10 LLM + ML cổ điển</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>cross-project</t>
+        </is>
+      </c>
+      <c r="W31" t="inlineStr">
+        <is>
+          <t>N (chia theo project)</t>
+        </is>
+      </c>
+      <c r="X31" t="inlineStr">
+        <is>
+          <t>không dùng</t>
+        </is>
+      </c>
+      <c r="Y31" t="inlineStr">
+        <is>
+          <t>P/R/F1</t>
+        </is>
+      </c>
+      <c r="Z31" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AA31" t="inlineStr">
+        <is>
+          <t>Y (replication package)</t>
+        </is>
+      </c>
+      <c r="AB31" t="inlineStr">
+        <is>
+          <t>mistral-nemo F1 0,62 (cross-project)</t>
+        </is>
+      </c>
+      <c r="AC31" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD31" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE31" t="n">
+        <v>2</v>
+      </c>
+      <c r="AF31" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG31" t="n">
+        <v>2</v>
+      </c>
       <c r="AH31">
         <f>IF(COUNT(AC31:AG31)=5,SUM(AC31:AG31),"")</f>
         <v/>
       </c>
       <c r="AI31" t="inlineStr"/>
-      <c r="AJ31" t="inlineStr"/>
+      <c r="AJ31" t="inlineStr">
+        <is>
+          <t>Nói thẳng: chia ngẫu nhiên có thể thổi phồng kết quả · Claude đọc (độ chắc chắn: cao)</t>
+        </is>
+      </c>
+      <c r="AK31" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -3839,9 +5487,21 @@
           <t>RQ3(a)</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr"/>
-      <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>15/26 chia ngẫu nhiên không khử trùng (R0007 R0018 R0060 R0125 R0187 R0406 R0517 R0538 R0617 R0618 R0625 R0632 R0655 R0719 R1202); 0/26 nhóm câu trùng khi chia; 5/26 không nêu cách chia</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>ĐỀ XUẤT: GAP CHÍNH (gộp với G2)</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Mạnh nhất: không bài nào kiểm soát câu trùng; Allamanis 2019 (R1526) cho thấy câu trùng thổi phồng metric tới 100% ở bài toán code</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -3889,9 +5549,21 @@
           <t>Mới (bổ sung RQ3)</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr"/>
-      <c r="K3" s="2" t="inlineStr"/>
-      <c r="L3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>7/26 dùng oversampling: 3 làm trước khi chia (R0187 R0538 R0632), 3 làm đúng trong train (R0181 R0517 R0719), 1 không rõ (R0618)</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>ĐỀ XUẤT: GAP CHÍNH (gộp với G1)</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Hai bài báo accuracy cao nhất bộ (R0632 98,79%, R0538 99%) đều oversampling trước khi chia; chưa bài nào đo mức thổi phồng</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -3939,9 +5611,21 @@
           <t>RQ1</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr"/>
-      <c r="L4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>6 bài ensemble: 4/6 không kiểm định (R0118 R0517 R0632 R1202); 2 bài có kiểm định (R0187 R0617) vẫn chia ngẫu nhiên không khử trùng</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>ĐỀ XUẤT: GAP PHỤ 1</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Câu hỏi: lợi thế ensemble có còn khi đánh giá có kiểm soát rò rỉ + kiểm định?</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -3989,8 +5673,16 @@
           <t>Hỗ trợ RQ1/RQ3</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr"/>
-      <c r="K5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Macro-F1: 1/26 (R0655); weighted: 4/26; chỉ accuracy: 5/26</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>ĐỀ XUẤT: không thành RQ, làm đóng góp phương pháp (báo cáo macro-F1 + theo lớp)</t>
+        </is>
+      </c>
       <c r="L5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
@@ -4039,9 +5731,21 @@
           <t>RQ3(b)</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="2" t="inlineStr"/>
-      <c r="L6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>4/26 đánh giá theo project / domain (R0164 R0637 R1341, R0181 leave-one-project-out)</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>ĐỀ XUẤT: GAP PHỤ 2 (nếu audit thấy PROMISE_exp đủ project)</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>R1341 nói thẳng chia ngẫu nhiên có thể thổi phồng kết quả</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -4089,8 +5793,16 @@
           <t>Hỗ trợ</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr"/>
-      <c r="K7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>5/26 công bố code/data (R0164 R0181 R0347 R0625 R1341)</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>ĐỀ XUẤT: không thành RQ, làm đóng góp (repo + dataset freeze)</t>
+        </is>
+      </c>
       <c r="L7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
@@ -4139,9 +5851,21 @@
           <t>RQ2</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr"/>
-      <c r="K8" s="2" t="inlineStr"/>
-      <c r="L8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>1/26 tách riêng ảnh hưởng tiền xử lý (R0125, Abad et al. 2017)</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>ĐỀ XUẤT: BỎ khỏi RQ chính (đã có Abad 2017); giữ P0 làm cấu hình mặc định</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Bỏ RQ2 tiền xử lý của v1.1 giúp giảm 2/3 số cấu hình</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>